<commit_message>
QPL Updates and Alternative Part Number added
</commit_message>
<xml_diff>
--- a/help.xlsx
+++ b/help.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230FC70D-A2A1-48E6-92AD-BDC882185FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05F9ABE0-56F5-4771-9958-345A1AD729D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="825" yWindow="540" windowWidth="27675" windowHeight="11790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3420" yWindow="3420" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
     <sheet name="Choicelists" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="140001" concurrentCalc="0"/>
+  <calcPr calcId="140001"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -102,7 +102,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="G3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -131,7 +131,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -159,7 +159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="I3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -183,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -211,7 +211,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="K3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -235,7 +235,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="L3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -259,7 +259,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="M3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -283,7 +283,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -307,7 +307,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
+    <comment ref="P3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -331,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
+    <comment ref="Q3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -356,7 +356,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
+    <comment ref="R3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -380,7 +380,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
+    <comment ref="S3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -404,7 +404,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
+    <comment ref="AH3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
       <text>
         <r>
           <rPr>
@@ -428,7 +428,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
+    <comment ref="AM3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
       <text>
         <r>
           <rPr>
@@ -457,7 +457,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="126">
   <si>
     <t>Participant / Manufacturer</t>
   </si>
@@ -861,6 +861,15 @@
   </si>
   <si>
     <t>Listing Date</t>
+  </si>
+  <si>
+    <t>Alternative Part Number</t>
+  </si>
+  <si>
+    <t>This is an optional field to enter any alternative part number associated with the pump being rated.  This field can be used to enter a third party model number or a different manufacturer’s model number for the same pump.</t>
+  </si>
+  <si>
+    <t>*  This field is optional and does not need to be filled out for the pump to be listed.</t>
   </si>
 </sst>
 </file>
@@ -2028,47 +2037,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AR13"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" customWidth="1"/>
-    <col min="4" max="4" width="52.140625" customWidth="1"/>
-    <col min="5" max="5" width="49.85546875" customWidth="1"/>
-    <col min="6" max="6" width="60.85546875" customWidth="1"/>
-    <col min="7" max="7" width="44.7109375" customWidth="1"/>
-    <col min="8" max="8" width="33.140625" customWidth="1"/>
-    <col min="9" max="9" width="73.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="63" customWidth="1"/>
-    <col min="11" max="11" width="37.85546875" customWidth="1"/>
-    <col min="12" max="13" width="34.7109375" customWidth="1"/>
-    <col min="14" max="14" width="29" customWidth="1"/>
-    <col min="15" max="15" width="25.85546875" customWidth="1"/>
-    <col min="16" max="16" width="39.7109375" customWidth="1"/>
-    <col min="17" max="17" width="54.140625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="11" style="1" customWidth="1"/>
-    <col min="19" max="21" width="11" customWidth="1"/>
-    <col min="22" max="22" width="11" style="3" customWidth="1"/>
-    <col min="23" max="23" width="11" customWidth="1"/>
-    <col min="24" max="24" width="11" style="1" customWidth="1"/>
-    <col min="25" max="25" width="11" style="5" customWidth="1"/>
-    <col min="26" max="26" width="11" style="4" customWidth="1"/>
-    <col min="27" max="27" width="11" customWidth="1"/>
-    <col min="28" max="28" width="11" style="3" customWidth="1"/>
-    <col min="29" max="29" width="11" style="1" customWidth="1"/>
-    <col min="30" max="31" width="11" customWidth="1"/>
-    <col min="32" max="32" width="11" style="3" customWidth="1"/>
-    <col min="33" max="33" width="39.7109375" style="1" customWidth="1"/>
-    <col min="34" max="34" width="11" style="1" customWidth="1"/>
-    <col min="35" max="36" width="11" customWidth="1"/>
-    <col min="37" max="37" width="11" style="3" customWidth="1"/>
-    <col min="38" max="38" width="50" style="2" customWidth="1"/>
-    <col min="39" max="39" width="18.7109375" style="2" customWidth="1"/>
-    <col min="40" max="42" width="18" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.109375" customWidth="1"/>
+    <col min="4" max="4" width="52.109375" customWidth="1"/>
+    <col min="5" max="6" width="49.88671875" customWidth="1"/>
+    <col min="7" max="7" width="60.88671875" customWidth="1"/>
+    <col min="8" max="8" width="44.6640625" customWidth="1"/>
+    <col min="9" max="9" width="33.109375" customWidth="1"/>
+    <col min="10" max="10" width="73.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="63" customWidth="1"/>
+    <col min="12" max="12" width="37.88671875" customWidth="1"/>
+    <col min="13" max="14" width="34.6640625" customWidth="1"/>
+    <col min="15" max="15" width="29" customWidth="1"/>
+    <col min="16" max="16" width="25.88671875" customWidth="1"/>
+    <col min="17" max="17" width="39.6640625" customWidth="1"/>
+    <col min="18" max="18" width="54.109375" style="2" customWidth="1"/>
+    <col min="19" max="19" width="11" style="1" customWidth="1"/>
+    <col min="20" max="22" width="11" customWidth="1"/>
+    <col min="23" max="23" width="11" style="3" customWidth="1"/>
+    <col min="24" max="24" width="11" customWidth="1"/>
+    <col min="25" max="25" width="11" style="1" customWidth="1"/>
+    <col min="26" max="26" width="11" style="5" customWidth="1"/>
+    <col min="27" max="27" width="11" style="4" customWidth="1"/>
+    <col min="28" max="28" width="11" customWidth="1"/>
+    <col min="29" max="29" width="11" style="3" customWidth="1"/>
+    <col min="30" max="30" width="11" style="1" customWidth="1"/>
+    <col min="31" max="32" width="11" customWidth="1"/>
+    <col min="33" max="33" width="11" style="3" customWidth="1"/>
+    <col min="34" max="34" width="39.6640625" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11" style="1" customWidth="1"/>
+    <col min="36" max="37" width="11" customWidth="1"/>
+    <col min="38" max="38" width="11" style="3" customWidth="1"/>
+    <col min="39" max="39" width="50" style="2" customWidth="1"/>
+    <col min="40" max="40" width="18.6640625" style="2" customWidth="1"/>
+    <col min="41" max="43" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="79" customFormat="1" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44" s="79" customFormat="1" ht="128.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="79" t="s">
         <v>88</v>
       </c>
@@ -2083,43 +2092,45 @@
         <v>72</v>
       </c>
       <c r="F1" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="G1" s="76" t="s">
         <v>93</v>
       </c>
-      <c r="G1" s="76" t="s">
+      <c r="H1" s="76" t="s">
         <v>74</v>
       </c>
-      <c r="H1" s="76" t="s">
+      <c r="I1" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="I1" s="76" t="s">
+      <c r="J1" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="J1" s="76" t="s">
+      <c r="K1" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="K1" s="76" t="s">
+      <c r="L1" s="76" t="s">
         <v>79</v>
       </c>
-      <c r="L1" s="76" t="s">
+      <c r="M1" s="76" t="s">
         <v>80</v>
       </c>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76" t="s">
+      <c r="N1" s="76"/>
+      <c r="O1" s="76" t="s">
         <v>82</v>
       </c>
-      <c r="O1" s="76" t="s">
+      <c r="P1" s="76" t="s">
         <v>83</v>
       </c>
-      <c r="P1" s="76" t="s">
+      <c r="Q1" s="76" t="s">
         <v>84</v>
       </c>
-      <c r="Q1" s="78" t="s">
+      <c r="R1" s="78" t="s">
         <v>85</v>
       </c>
-      <c r="R1" s="97" t="s">
+      <c r="S1" s="97" t="s">
         <v>90</v>
       </c>
-      <c r="S1" s="98"/>
       <c r="T1" s="98"/>
       <c r="U1" s="98"/>
       <c r="V1" s="98"/>
@@ -2132,25 +2143,26 @@
       <c r="AC1" s="98"/>
       <c r="AD1" s="98"/>
       <c r="AE1" s="98"/>
-      <c r="AF1" s="99"/>
-      <c r="AG1" s="77" t="s">
+      <c r="AF1" s="98"/>
+      <c r="AG1" s="99"/>
+      <c r="AH1" s="77" t="s">
         <v>94</v>
       </c>
-      <c r="AH1" s="97" t="s">
+      <c r="AI1" s="97" t="s">
         <v>96</v>
       </c>
-      <c r="AI1" s="98"/>
       <c r="AJ1" s="98"/>
-      <c r="AK1" s="99"/>
-      <c r="AL1" s="78" t="s">
+      <c r="AK1" s="98"/>
+      <c r="AL1" s="99"/>
+      <c r="AM1" s="78" t="s">
         <v>97</v>
       </c>
-      <c r="AM1" s="80"/>
-      <c r="AN1" s="81"/>
-      <c r="AP1" s="80"/>
+      <c r="AN1" s="80"/>
+      <c r="AO1" s="81"/>
       <c r="AQ1" s="80"/>
+      <c r="AR1" s="80"/>
     </row>
-    <row r="2" spans="1:43" s="76" customFormat="1" ht="76.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:44" s="76" customFormat="1" ht="76.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="76" t="s">
         <v>89</v>
       </c>
@@ -2166,11 +2178,13 @@
       <c r="E2" s="75" t="s">
         <v>86</v>
       </c>
-      <c r="Q2" s="78"/>
-      <c r="R2" s="94" t="s">
+      <c r="F2" s="75" t="s">
+        <v>125</v>
+      </c>
+      <c r="R2" s="78"/>
+      <c r="S2" s="94" t="s">
         <v>92</v>
       </c>
-      <c r="S2" s="95"/>
       <c r="T2" s="95"/>
       <c r="U2" s="95"/>
       <c r="V2" s="95"/>
@@ -2183,26 +2197,27 @@
       <c r="AC2" s="95"/>
       <c r="AD2" s="95"/>
       <c r="AE2" s="95"/>
-      <c r="AF2" s="96"/>
-      <c r="AG2" s="77" t="s">
+      <c r="AF2" s="95"/>
+      <c r="AG2" s="96"/>
+      <c r="AH2" s="77" t="s">
         <v>95</v>
       </c>
-      <c r="AH2" s="94" t="s">
+      <c r="AI2" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="AI2" s="95"/>
       <c r="AJ2" s="95"/>
-      <c r="AK2" s="96"/>
-      <c r="AL2" s="78" t="s">
+      <c r="AK2" s="95"/>
+      <c r="AL2" s="96"/>
+      <c r="AM2" s="78" t="s">
         <v>87</v>
       </c>
-      <c r="AM2" s="77"/>
-      <c r="AN2" s="93"/>
+      <c r="AN2" s="77"/>
       <c r="AO2" s="93"/>
       <c r="AP2" s="93"/>
-      <c r="AQ2" s="77"/>
+      <c r="AQ2" s="93"/>
+      <c r="AR2" s="77"/>
     </row>
-    <row r="3" spans="1:43" s="6" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:44" s="6" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
@@ -2216,177 +2231,178 @@
         <v>3</v>
       </c>
       <c r="F3" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="M3" s="87" t="s">
+      <c r="N3" s="87" t="s">
         <v>114</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="P3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="Q3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="11" t="s">
+      <c r="R3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="S3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="S3" s="13" t="s">
+      <c r="T3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="T3" s="13" t="s">
+      <c r="U3" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="U3" s="14" t="s">
+      <c r="V3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="V3" s="15" t="s">
+      <c r="W3" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="W3" s="16" t="s">
+      <c r="X3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="X3" s="17" t="s">
+      <c r="Y3" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="Y3" s="18" t="s">
+      <c r="Z3" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="Z3" s="19" t="s">
+      <c r="AA3" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="AA3" s="20" t="s">
+      <c r="AB3" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="AB3" s="21" t="s">
+      <c r="AC3" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="AC3" s="22" t="s">
+      <c r="AD3" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="AD3" s="23" t="s">
+      <c r="AE3" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="AE3" s="23" t="s">
+      <c r="AF3" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="AF3" s="24" t="s">
+      <c r="AG3" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="AG3" s="25" t="s">
+      <c r="AH3" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="AH3" s="26" t="s">
+      <c r="AI3" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="AI3" s="27" t="s">
+      <c r="AJ3" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="AJ3" s="27" t="s">
+      <c r="AK3" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="AK3" s="28" t="s">
+      <c r="AL3" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="AL3" s="29" t="s">
+      <c r="AM3" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="AM3" s="30" t="s">
+      <c r="AN3" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="AN3" s="90" t="s">
+      <c r="AO3" s="90" t="s">
         <v>120</v>
       </c>
-      <c r="AO3" s="90" t="s">
+      <c r="AP3" s="90" t="s">
         <v>121</v>
       </c>
-      <c r="AP3" s="90" t="s">
+      <c r="AQ3" s="90" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:43" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:44" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="32"/>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
       <c r="E4" s="32"/>
       <c r="F4" s="32"/>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="32"/>
+      <c r="H4" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="32"/>
       <c r="I4" s="32"/>
       <c r="J4" s="32"/>
       <c r="K4" s="32"/>
       <c r="L4" s="32"/>
-      <c r="M4" s="33" t="s">
+      <c r="M4" s="32"/>
+      <c r="N4" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="N4" s="32" t="s">
+      <c r="O4" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="O4" s="32" t="s">
+      <c r="P4" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="P4" s="32"/>
-      <c r="Q4" s="34" t="s">
+      <c r="Q4" s="32"/>
+      <c r="R4" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="R4" s="107" t="s">
+      <c r="S4" s="107" t="s">
         <v>81</v>
       </c>
-      <c r="S4" s="108"/>
       <c r="T4" s="108"/>
       <c r="U4" s="108"/>
-      <c r="V4" s="109"/>
-      <c r="W4" s="35"/>
-      <c r="X4" s="102" t="s">
+      <c r="V4" s="108"/>
+      <c r="W4" s="109"/>
+      <c r="X4" s="35"/>
+      <c r="Y4" s="102" t="s">
         <v>68</v>
       </c>
-      <c r="Y4" s="102"/>
       <c r="Z4" s="102"/>
       <c r="AA4" s="102"/>
       <c r="AB4" s="102"/>
-      <c r="AC4" s="103" t="s">
+      <c r="AC4" s="102"/>
+      <c r="AD4" s="103" t="s">
         <v>69</v>
       </c>
-      <c r="AD4" s="103"/>
       <c r="AE4" s="103"/>
       <c r="AF4" s="103"/>
-      <c r="AG4" s="38"/>
-      <c r="AH4" s="39"/>
-      <c r="AI4" s="40"/>
+      <c r="AG4" s="103"/>
+      <c r="AH4" s="38"/>
+      <c r="AI4" s="39"/>
       <c r="AJ4" s="40"/>
-      <c r="AK4" s="41"/>
-      <c r="AL4" s="42" t="s">
+      <c r="AK4" s="40"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="AM4" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="AN4" s="91" t="s">
+      <c r="AN4" s="43" t="s">
         <v>40</v>
       </c>
       <c r="AO4" s="91" t="s">
@@ -2395,8 +2411,11 @@
       <c r="AP4" s="91" t="s">
         <v>40</v>
       </c>
+      <c r="AQ4" s="91" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="5" spans="1:43" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:44" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="45" t="s">
         <v>98</v>
       </c>
@@ -2409,69 +2428,70 @@
       <c r="E5" s="46" t="s">
         <v>101</v>
       </c>
-      <c r="F5" s="46" t="s">
+      <c r="F5" s="46"/>
+      <c r="G5" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="G5" s="46"/>
-      <c r="H5" s="46" t="s">
+      <c r="H5" s="46"/>
+      <c r="I5" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="I5" s="46"/>
-      <c r="J5" s="46" t="s">
+      <c r="J5" s="46"/>
+      <c r="K5" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="K5" s="46" t="s">
+      <c r="L5" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="L5" s="46" t="s">
+      <c r="M5" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="M5" s="46"/>
-      <c r="N5" s="46" t="s">
+      <c r="N5" s="46"/>
+      <c r="O5" s="46" t="s">
         <v>108</v>
       </c>
-      <c r="O5" s="47" t="s">
+      <c r="P5" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="P5" s="46" t="s">
+      <c r="Q5" s="46" t="s">
         <v>107</v>
       </c>
-      <c r="Q5" s="34" t="s">
+      <c r="R5" s="34" t="s">
         <v>110</v>
       </c>
-      <c r="R5" s="82" t="s">
+      <c r="S5" s="82" t="s">
         <v>112</v>
       </c>
-      <c r="S5" s="83"/>
       <c r="T5" s="83"/>
       <c r="U5" s="83"/>
       <c r="V5" s="83"/>
-      <c r="W5" s="35"/>
-      <c r="X5" s="84"/>
-      <c r="Y5" s="85"/>
+      <c r="W5" s="83"/>
+      <c r="X5" s="35"/>
+      <c r="Y5" s="84"/>
       <c r="Z5" s="85"/>
       <c r="AA5" s="85"/>
       <c r="AB5" s="85"/>
-      <c r="AC5" s="86"/>
+      <c r="AC5" s="85"/>
       <c r="AD5" s="86"/>
       <c r="AE5" s="86"/>
       <c r="AF5" s="86"/>
-      <c r="AG5" s="38" t="s">
+      <c r="AG5" s="86"/>
+      <c r="AH5" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="AH5" s="36"/>
-      <c r="AI5" s="37"/>
+      <c r="AI5" s="36"/>
       <c r="AJ5" s="37"/>
       <c r="AK5" s="37"/>
-      <c r="AL5" s="42" t="s">
+      <c r="AL5" s="37"/>
+      <c r="AM5" s="42" t="s">
         <v>105</v>
       </c>
-      <c r="AM5" s="43"/>
-      <c r="AN5" s="92"/>
+      <c r="AN5" s="43"/>
       <c r="AO5" s="92"/>
       <c r="AP5" s="92"/>
+      <c r="AQ5" s="92"/>
     </row>
-    <row r="6" spans="1:43" s="44" customFormat="1" ht="83.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:44" s="44" customFormat="1" ht="83.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="45" t="s">
         <v>98</v>
       </c>
@@ -2486,87 +2506,86 @@
       </c>
       <c r="F6" s="46"/>
       <c r="G6" s="46"/>
-      <c r="H6" s="46" t="s">
+      <c r="H6" s="46"/>
+      <c r="I6" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46" t="s">
+      <c r="J6" s="46"/>
+      <c r="K6" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="K6" s="46" t="s">
+      <c r="L6" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="L6" s="46"/>
-      <c r="M6" s="55"/>
-      <c r="N6" s="46"/>
-      <c r="O6" s="47"/>
-      <c r="P6" s="46"/>
-      <c r="Q6" s="48" t="s">
+      <c r="M6" s="46"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="46"/>
+      <c r="P6" s="47"/>
+      <c r="Q6" s="46"/>
+      <c r="R6" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="R6" s="104" t="s">
+      <c r="S6" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="S6" s="104"/>
       <c r="T6" s="104"/>
       <c r="U6" s="104"/>
       <c r="V6" s="104"/>
-      <c r="W6" s="49"/>
-      <c r="X6" s="50"/>
-      <c r="Y6" s="105" t="s">
+      <c r="W6" s="104"/>
+      <c r="X6" s="49"/>
+      <c r="Y6" s="50"/>
+      <c r="Z6" s="105" t="s">
         <v>43</v>
       </c>
-      <c r="Z6" s="105"/>
-      <c r="AA6" s="105" t="s">
+      <c r="AA6" s="105"/>
+      <c r="AB6" s="105" t="s">
         <v>44</v>
       </c>
-      <c r="AB6" s="105"/>
-      <c r="AC6" s="106"/>
+      <c r="AC6" s="105"/>
       <c r="AD6" s="106"/>
       <c r="AE6" s="106"/>
       <c r="AF6" s="106"/>
-      <c r="AG6" s="51"/>
-      <c r="AH6" s="100" t="s">
+      <c r="AG6" s="106"/>
+      <c r="AH6" s="51"/>
+      <c r="AI6" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="AI6" s="100"/>
-      <c r="AJ6" s="101" t="s">
+      <c r="AJ6" s="100"/>
+      <c r="AK6" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="AK6" s="101"/>
-      <c r="AL6" s="52"/>
-      <c r="AM6" s="53"/>
-      <c r="AN6" s="92"/>
+      <c r="AL6" s="101"/>
+      <c r="AM6" s="52"/>
+      <c r="AN6" s="53"/>
       <c r="AO6" s="92"/>
       <c r="AP6" s="92"/>
+      <c r="AQ6" s="92"/>
     </row>
-    <row r="7" spans="1:43" s="54" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:44" s="54" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="55"/>
       <c r="C7" s="55"/>
       <c r="D7" s="55"/>
       <c r="E7" s="55"/>
       <c r="F7" s="55"/>
       <c r="G7" s="55"/>
-      <c r="H7" s="55" t="s">
+      <c r="H7" s="55"/>
+      <c r="I7" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="55"/>
       <c r="J7" s="55"/>
       <c r="K7" s="55"/>
-      <c r="L7" s="55" t="s">
+      <c r="L7" s="55"/>
+      <c r="M7" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="55"/>
       <c r="N7" s="55"/>
-      <c r="O7" s="56"/>
-      <c r="P7" s="56" t="s">
+      <c r="O7" s="55"/>
+      <c r="P7" s="56"/>
+      <c r="Q7" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="58" t="s">
-        <v>47</v>
-      </c>
-      <c r="S7" s="59" t="s">
+      <c r="R7" s="57"/>
+      <c r="S7" s="58" t="s">
         <v>47</v>
       </c>
       <c r="T7" s="59" t="s">
@@ -2575,16 +2594,16 @@
       <c r="U7" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="V7" s="60" t="s">
+      <c r="V7" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="W7" s="61" t="s">
+      <c r="W7" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="X7" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="X7" s="64" t="s">
-        <v>46</v>
-      </c>
-      <c r="Y7" s="65" t="s">
+      <c r="Y7" s="64" t="s">
         <v>46</v>
       </c>
       <c r="Z7" s="65" t="s">
@@ -2593,13 +2612,13 @@
       <c r="AA7" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="AB7" s="66" t="s">
+      <c r="AB7" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="AC7" s="67" t="s">
+      <c r="AC7" s="66" t="s">
         <v>46</v>
       </c>
-      <c r="AD7" s="68" t="s">
+      <c r="AD7" s="67" t="s">
         <v>46</v>
       </c>
       <c r="AE7" s="68" t="s">
@@ -2608,23 +2627,26 @@
       <c r="AF7" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="AG7" s="69"/>
-      <c r="AH7" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI7" s="63" t="s">
+      <c r="AG7" s="68" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH7" s="69"/>
+      <c r="AI7" s="62" t="s">
         <v>48</v>
       </c>
       <c r="AJ7" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="AK7" s="70" t="s">
+      <c r="AK7" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="AL7" s="71"/>
-      <c r="AM7" s="72"/>
+      <c r="AL7" s="70" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM7" s="71"/>
+      <c r="AN7" s="72"/>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>49</v>
       </c>
@@ -2637,66 +2659,66 @@
       <c r="E8" t="s">
         <v>61</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>58</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>10</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>5</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>1</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>3600</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>59</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>95</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>60</v>
       </c>
-      <c r="Q8" s="2" t="s">
+      <c r="R8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R8" s="1">
+      <c r="S8" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <v>424.4298</v>
       </c>
-      <c r="X8" s="1">
+      <c r="Y8" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y8" s="5">
+      <c r="Z8" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z8" s="4">
+      <c r="AA8" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG8" s="1">
+      <c r="AH8" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH8" s="1">
+      <c r="AI8" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI8">
+      <c r="AJ8">
         <v>383.476</v>
       </c>
-      <c r="AK8" s="73"/>
-      <c r="AL8" s="2">
+      <c r="AL8" s="73"/>
+      <c r="AM8" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
@@ -2709,65 +2731,65 @@
       <c r="E9" t="s">
         <v>62</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>57</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>58</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>10</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>5</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>1</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>3600</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>59</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>96</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>60</v>
       </c>
-      <c r="Q9" s="2" t="s">
+      <c r="R9" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R9" s="1">
+      <c r="S9" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <v>424.4298</v>
       </c>
-      <c r="X9" s="1">
+      <c r="Y9" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y9" s="5">
+      <c r="Z9" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z9" s="4">
+      <c r="AA9" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG9" s="1">
+      <c r="AH9" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH9" s="1">
+      <c r="AI9" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI9">
+      <c r="AJ9">
         <v>383.476</v>
       </c>
-      <c r="AL9" s="2">
+      <c r="AM9" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>49</v>
       </c>
@@ -2780,65 +2802,65 @@
       <c r="E10" t="s">
         <v>63</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>57</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>58</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>10</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>5</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>1</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>3600</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>59</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>97</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>60</v>
       </c>
-      <c r="Q10" s="2" t="s">
+      <c r="R10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R10" s="1">
+      <c r="S10" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <v>424.4298</v>
       </c>
-      <c r="X10" s="1">
+      <c r="Y10" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y10" s="5">
+      <c r="Z10" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z10" s="4">
+      <c r="AA10" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG10" s="1">
+      <c r="AH10" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH10" s="1">
+      <c r="AI10" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI10">
+      <c r="AJ10">
         <v>383.476</v>
       </c>
-      <c r="AL10" s="2">
+      <c r="AM10" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>49</v>
       </c>
@@ -2851,65 +2873,65 @@
       <c r="E11" t="s">
         <v>64</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>57</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>58</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>10</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>5</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>1</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>3600</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>59</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>95</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>75</v>
       </c>
-      <c r="Q11" s="2" t="s">
+      <c r="R11" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R11" s="1">
+      <c r="S11" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W11">
+      <c r="X11">
         <v>424.4298</v>
       </c>
-      <c r="X11" s="1">
+      <c r="Y11" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y11" s="5">
+      <c r="Z11" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z11" s="4">
+      <c r="AA11" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG11" s="1">
+      <c r="AH11" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH11" s="1">
+      <c r="AI11" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI11">
+      <c r="AJ11">
         <v>383.476</v>
       </c>
-      <c r="AL11" s="2">
+      <c r="AM11" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>49</v>
       </c>
@@ -2922,68 +2944,68 @@
       <c r="E12" t="s">
         <v>65</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>57</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>58</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>10</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>5</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>1</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>3600</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>59</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>96</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>75</v>
       </c>
-      <c r="Q12" s="2" t="s">
+      <c r="R12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R12" s="1">
+      <c r="S12" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W12">
+      <c r="X12">
         <v>424.4298</v>
       </c>
-      <c r="X12" s="1">
+      <c r="Y12" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y12" s="5">
+      <c r="Z12" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z12" s="4">
+      <c r="AA12" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG12" s="1">
+      <c r="AH12" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH12" s="1">
+      <c r="AI12" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI12">
+      <c r="AJ12">
         <v>383.476</v>
       </c>
-      <c r="AJ12" t="s">
+      <c r="AK12" t="s">
         <v>52</v>
       </c>
-      <c r="AL12" s="2">
+      <c r="AM12" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>49</v>
       </c>
@@ -2996,79 +3018,79 @@
       <c r="E13" t="s">
         <v>66</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>57</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>58</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>10</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>5</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>1</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>3600</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>59</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>97</v>
       </c>
-      <c r="P13">
+      <c r="Q13">
         <v>75</v>
       </c>
-      <c r="Q13" s="2" t="s">
+      <c r="R13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R13" s="1">
+      <c r="S13" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W13">
+      <c r="X13">
         <v>424.4298</v>
       </c>
-      <c r="X13" s="1">
+      <c r="Y13" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y13" s="5">
+      <c r="Z13" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z13" s="4">
+      <c r="AA13" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG13" s="1">
+      <c r="AH13" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH13" s="1">
+      <c r="AI13" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI13">
+      <c r="AJ13">
         <v>383.476</v>
       </c>
-      <c r="AL13" s="2">
+      <c r="AM13" s="2">
         <v>106</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="AH2:AK2"/>
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="R1:AF1"/>
-    <mergeCell ref="R2:AF2"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="X4:AB4"/>
-    <mergeCell ref="AC4:AF4"/>
-    <mergeCell ref="R6:V6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="AC6:AF6"/>
-    <mergeCell ref="R4:V4"/>
+    <mergeCell ref="AI2:AL2"/>
+    <mergeCell ref="AI1:AL1"/>
+    <mergeCell ref="S1:AG1"/>
+    <mergeCell ref="S2:AG2"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="Y4:AC4"/>
+    <mergeCell ref="AD4:AG4"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AD6:AG6"/>
+    <mergeCell ref="S4:W4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
@@ -3084,49 +3106,49 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="88" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="74" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="74" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="74" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="74" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="89" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>119</v>
       </c>

</xml_diff>

<commit_message>
3-2026 QPL, Alt Model Number changes (#23)
* QPL Updates and Alternative Part Number added

* More
</commit_message>
<xml_diff>
--- a/help.xlsx
+++ b/help.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230FC70D-A2A1-48E6-92AD-BDC882185FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05F9ABE0-56F5-4771-9958-345A1AD729D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="825" yWindow="540" windowWidth="27675" windowHeight="11790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3420" yWindow="3420" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
     <sheet name="Choicelists" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="140001" concurrentCalc="0"/>
+  <calcPr calcId="140001"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -102,7 +102,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="G3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -131,7 +131,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -159,7 +159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="I3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -183,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -211,7 +211,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="K3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -235,7 +235,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="L3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -259,7 +259,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="M3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -283,7 +283,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -307,7 +307,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
+    <comment ref="P3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -331,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
+    <comment ref="Q3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -356,7 +356,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
+    <comment ref="R3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -380,7 +380,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
+    <comment ref="S3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -404,7 +404,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
+    <comment ref="AH3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
       <text>
         <r>
           <rPr>
@@ -428,7 +428,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
+    <comment ref="AM3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
       <text>
         <r>
           <rPr>
@@ -457,7 +457,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="126">
   <si>
     <t>Participant / Manufacturer</t>
   </si>
@@ -861,6 +861,15 @@
   </si>
   <si>
     <t>Listing Date</t>
+  </si>
+  <si>
+    <t>Alternative Part Number</t>
+  </si>
+  <si>
+    <t>This is an optional field to enter any alternative part number associated with the pump being rated.  This field can be used to enter a third party model number or a different manufacturer’s model number for the same pump.</t>
+  </si>
+  <si>
+    <t>*  This field is optional and does not need to be filled out for the pump to be listed.</t>
   </si>
 </sst>
 </file>
@@ -2028,47 +2037,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AR13"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" customWidth="1"/>
-    <col min="4" max="4" width="52.140625" customWidth="1"/>
-    <col min="5" max="5" width="49.85546875" customWidth="1"/>
-    <col min="6" max="6" width="60.85546875" customWidth="1"/>
-    <col min="7" max="7" width="44.7109375" customWidth="1"/>
-    <col min="8" max="8" width="33.140625" customWidth="1"/>
-    <col min="9" max="9" width="73.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="63" customWidth="1"/>
-    <col min="11" max="11" width="37.85546875" customWidth="1"/>
-    <col min="12" max="13" width="34.7109375" customWidth="1"/>
-    <col min="14" max="14" width="29" customWidth="1"/>
-    <col min="15" max="15" width="25.85546875" customWidth="1"/>
-    <col min="16" max="16" width="39.7109375" customWidth="1"/>
-    <col min="17" max="17" width="54.140625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="11" style="1" customWidth="1"/>
-    <col min="19" max="21" width="11" customWidth="1"/>
-    <col min="22" max="22" width="11" style="3" customWidth="1"/>
-    <col min="23" max="23" width="11" customWidth="1"/>
-    <col min="24" max="24" width="11" style="1" customWidth="1"/>
-    <col min="25" max="25" width="11" style="5" customWidth="1"/>
-    <col min="26" max="26" width="11" style="4" customWidth="1"/>
-    <col min="27" max="27" width="11" customWidth="1"/>
-    <col min="28" max="28" width="11" style="3" customWidth="1"/>
-    <col min="29" max="29" width="11" style="1" customWidth="1"/>
-    <col min="30" max="31" width="11" customWidth="1"/>
-    <col min="32" max="32" width="11" style="3" customWidth="1"/>
-    <col min="33" max="33" width="39.7109375" style="1" customWidth="1"/>
-    <col min="34" max="34" width="11" style="1" customWidth="1"/>
-    <col min="35" max="36" width="11" customWidth="1"/>
-    <col min="37" max="37" width="11" style="3" customWidth="1"/>
-    <col min="38" max="38" width="50" style="2" customWidth="1"/>
-    <col min="39" max="39" width="18.7109375" style="2" customWidth="1"/>
-    <col min="40" max="42" width="18" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.109375" customWidth="1"/>
+    <col min="4" max="4" width="52.109375" customWidth="1"/>
+    <col min="5" max="6" width="49.88671875" customWidth="1"/>
+    <col min="7" max="7" width="60.88671875" customWidth="1"/>
+    <col min="8" max="8" width="44.6640625" customWidth="1"/>
+    <col min="9" max="9" width="33.109375" customWidth="1"/>
+    <col min="10" max="10" width="73.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="63" customWidth="1"/>
+    <col min="12" max="12" width="37.88671875" customWidth="1"/>
+    <col min="13" max="14" width="34.6640625" customWidth="1"/>
+    <col min="15" max="15" width="29" customWidth="1"/>
+    <col min="16" max="16" width="25.88671875" customWidth="1"/>
+    <col min="17" max="17" width="39.6640625" customWidth="1"/>
+    <col min="18" max="18" width="54.109375" style="2" customWidth="1"/>
+    <col min="19" max="19" width="11" style="1" customWidth="1"/>
+    <col min="20" max="22" width="11" customWidth="1"/>
+    <col min="23" max="23" width="11" style="3" customWidth="1"/>
+    <col min="24" max="24" width="11" customWidth="1"/>
+    <col min="25" max="25" width="11" style="1" customWidth="1"/>
+    <col min="26" max="26" width="11" style="5" customWidth="1"/>
+    <col min="27" max="27" width="11" style="4" customWidth="1"/>
+    <col min="28" max="28" width="11" customWidth="1"/>
+    <col min="29" max="29" width="11" style="3" customWidth="1"/>
+    <col min="30" max="30" width="11" style="1" customWidth="1"/>
+    <col min="31" max="32" width="11" customWidth="1"/>
+    <col min="33" max="33" width="11" style="3" customWidth="1"/>
+    <col min="34" max="34" width="39.6640625" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11" style="1" customWidth="1"/>
+    <col min="36" max="37" width="11" customWidth="1"/>
+    <col min="38" max="38" width="11" style="3" customWidth="1"/>
+    <col min="39" max="39" width="50" style="2" customWidth="1"/>
+    <col min="40" max="40" width="18.6640625" style="2" customWidth="1"/>
+    <col min="41" max="43" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="79" customFormat="1" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44" s="79" customFormat="1" ht="128.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="79" t="s">
         <v>88</v>
       </c>
@@ -2083,43 +2092,45 @@
         <v>72</v>
       </c>
       <c r="F1" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="G1" s="76" t="s">
         <v>93</v>
       </c>
-      <c r="G1" s="76" t="s">
+      <c r="H1" s="76" t="s">
         <v>74</v>
       </c>
-      <c r="H1" s="76" t="s">
+      <c r="I1" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="I1" s="76" t="s">
+      <c r="J1" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="J1" s="76" t="s">
+      <c r="K1" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="K1" s="76" t="s">
+      <c r="L1" s="76" t="s">
         <v>79</v>
       </c>
-      <c r="L1" s="76" t="s">
+      <c r="M1" s="76" t="s">
         <v>80</v>
       </c>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76" t="s">
+      <c r="N1" s="76"/>
+      <c r="O1" s="76" t="s">
         <v>82</v>
       </c>
-      <c r="O1" s="76" t="s">
+      <c r="P1" s="76" t="s">
         <v>83</v>
       </c>
-      <c r="P1" s="76" t="s">
+      <c r="Q1" s="76" t="s">
         <v>84</v>
       </c>
-      <c r="Q1" s="78" t="s">
+      <c r="R1" s="78" t="s">
         <v>85</v>
       </c>
-      <c r="R1" s="97" t="s">
+      <c r="S1" s="97" t="s">
         <v>90</v>
       </c>
-      <c r="S1" s="98"/>
       <c r="T1" s="98"/>
       <c r="U1" s="98"/>
       <c r="V1" s="98"/>
@@ -2132,25 +2143,26 @@
       <c r="AC1" s="98"/>
       <c r="AD1" s="98"/>
       <c r="AE1" s="98"/>
-      <c r="AF1" s="99"/>
-      <c r="AG1" s="77" t="s">
+      <c r="AF1" s="98"/>
+      <c r="AG1" s="99"/>
+      <c r="AH1" s="77" t="s">
         <v>94</v>
       </c>
-      <c r="AH1" s="97" t="s">
+      <c r="AI1" s="97" t="s">
         <v>96</v>
       </c>
-      <c r="AI1" s="98"/>
       <c r="AJ1" s="98"/>
-      <c r="AK1" s="99"/>
-      <c r="AL1" s="78" t="s">
+      <c r="AK1" s="98"/>
+      <c r="AL1" s="99"/>
+      <c r="AM1" s="78" t="s">
         <v>97</v>
       </c>
-      <c r="AM1" s="80"/>
-      <c r="AN1" s="81"/>
-      <c r="AP1" s="80"/>
+      <c r="AN1" s="80"/>
+      <c r="AO1" s="81"/>
       <c r="AQ1" s="80"/>
+      <c r="AR1" s="80"/>
     </row>
-    <row r="2" spans="1:43" s="76" customFormat="1" ht="76.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:44" s="76" customFormat="1" ht="76.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="76" t="s">
         <v>89</v>
       </c>
@@ -2166,11 +2178,13 @@
       <c r="E2" s="75" t="s">
         <v>86</v>
       </c>
-      <c r="Q2" s="78"/>
-      <c r="R2" s="94" t="s">
+      <c r="F2" s="75" t="s">
+        <v>125</v>
+      </c>
+      <c r="R2" s="78"/>
+      <c r="S2" s="94" t="s">
         <v>92</v>
       </c>
-      <c r="S2" s="95"/>
       <c r="T2" s="95"/>
       <c r="U2" s="95"/>
       <c r="V2" s="95"/>
@@ -2183,26 +2197,27 @@
       <c r="AC2" s="95"/>
       <c r="AD2" s="95"/>
       <c r="AE2" s="95"/>
-      <c r="AF2" s="96"/>
-      <c r="AG2" s="77" t="s">
+      <c r="AF2" s="95"/>
+      <c r="AG2" s="96"/>
+      <c r="AH2" s="77" t="s">
         <v>95</v>
       </c>
-      <c r="AH2" s="94" t="s">
+      <c r="AI2" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="AI2" s="95"/>
       <c r="AJ2" s="95"/>
-      <c r="AK2" s="96"/>
-      <c r="AL2" s="78" t="s">
+      <c r="AK2" s="95"/>
+      <c r="AL2" s="96"/>
+      <c r="AM2" s="78" t="s">
         <v>87</v>
       </c>
-      <c r="AM2" s="77"/>
-      <c r="AN2" s="93"/>
+      <c r="AN2" s="77"/>
       <c r="AO2" s="93"/>
       <c r="AP2" s="93"/>
-      <c r="AQ2" s="77"/>
+      <c r="AQ2" s="93"/>
+      <c r="AR2" s="77"/>
     </row>
-    <row r="3" spans="1:43" s="6" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:44" s="6" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
@@ -2216,177 +2231,178 @@
         <v>3</v>
       </c>
       <c r="F3" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="M3" s="87" t="s">
+      <c r="N3" s="87" t="s">
         <v>114</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="P3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="Q3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="11" t="s">
+      <c r="R3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="S3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="S3" s="13" t="s">
+      <c r="T3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="T3" s="13" t="s">
+      <c r="U3" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="U3" s="14" t="s">
+      <c r="V3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="V3" s="15" t="s">
+      <c r="W3" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="W3" s="16" t="s">
+      <c r="X3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="X3" s="17" t="s">
+      <c r="Y3" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="Y3" s="18" t="s">
+      <c r="Z3" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="Z3" s="19" t="s">
+      <c r="AA3" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="AA3" s="20" t="s">
+      <c r="AB3" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="AB3" s="21" t="s">
+      <c r="AC3" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="AC3" s="22" t="s">
+      <c r="AD3" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="AD3" s="23" t="s">
+      <c r="AE3" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="AE3" s="23" t="s">
+      <c r="AF3" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="AF3" s="24" t="s">
+      <c r="AG3" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="AG3" s="25" t="s">
+      <c r="AH3" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="AH3" s="26" t="s">
+      <c r="AI3" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="AI3" s="27" t="s">
+      <c r="AJ3" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="AJ3" s="27" t="s">
+      <c r="AK3" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="AK3" s="28" t="s">
+      <c r="AL3" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="AL3" s="29" t="s">
+      <c r="AM3" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="AM3" s="30" t="s">
+      <c r="AN3" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="AN3" s="90" t="s">
+      <c r="AO3" s="90" t="s">
         <v>120</v>
       </c>
-      <c r="AO3" s="90" t="s">
+      <c r="AP3" s="90" t="s">
         <v>121</v>
       </c>
-      <c r="AP3" s="90" t="s">
+      <c r="AQ3" s="90" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:43" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:44" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="32"/>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
       <c r="E4" s="32"/>
       <c r="F4" s="32"/>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="32"/>
+      <c r="H4" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="32"/>
       <c r="I4" s="32"/>
       <c r="J4" s="32"/>
       <c r="K4" s="32"/>
       <c r="L4" s="32"/>
-      <c r="M4" s="33" t="s">
+      <c r="M4" s="32"/>
+      <c r="N4" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="N4" s="32" t="s">
+      <c r="O4" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="O4" s="32" t="s">
+      <c r="P4" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="P4" s="32"/>
-      <c r="Q4" s="34" t="s">
+      <c r="Q4" s="32"/>
+      <c r="R4" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="R4" s="107" t="s">
+      <c r="S4" s="107" t="s">
         <v>81</v>
       </c>
-      <c r="S4" s="108"/>
       <c r="T4" s="108"/>
       <c r="U4" s="108"/>
-      <c r="V4" s="109"/>
-      <c r="W4" s="35"/>
-      <c r="X4" s="102" t="s">
+      <c r="V4" s="108"/>
+      <c r="W4" s="109"/>
+      <c r="X4" s="35"/>
+      <c r="Y4" s="102" t="s">
         <v>68</v>
       </c>
-      <c r="Y4" s="102"/>
       <c r="Z4" s="102"/>
       <c r="AA4" s="102"/>
       <c r="AB4" s="102"/>
-      <c r="AC4" s="103" t="s">
+      <c r="AC4" s="102"/>
+      <c r="AD4" s="103" t="s">
         <v>69</v>
       </c>
-      <c r="AD4" s="103"/>
       <c r="AE4" s="103"/>
       <c r="AF4" s="103"/>
-      <c r="AG4" s="38"/>
-      <c r="AH4" s="39"/>
-      <c r="AI4" s="40"/>
+      <c r="AG4" s="103"/>
+      <c r="AH4" s="38"/>
+      <c r="AI4" s="39"/>
       <c r="AJ4" s="40"/>
-      <c r="AK4" s="41"/>
-      <c r="AL4" s="42" t="s">
+      <c r="AK4" s="40"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="AM4" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="AN4" s="91" t="s">
+      <c r="AN4" s="43" t="s">
         <v>40</v>
       </c>
       <c r="AO4" s="91" t="s">
@@ -2395,8 +2411,11 @@
       <c r="AP4" s="91" t="s">
         <v>40</v>
       </c>
+      <c r="AQ4" s="91" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="5" spans="1:43" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:44" s="31" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="45" t="s">
         <v>98</v>
       </c>
@@ -2409,69 +2428,70 @@
       <c r="E5" s="46" t="s">
         <v>101</v>
       </c>
-      <c r="F5" s="46" t="s">
+      <c r="F5" s="46"/>
+      <c r="G5" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="G5" s="46"/>
-      <c r="H5" s="46" t="s">
+      <c r="H5" s="46"/>
+      <c r="I5" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="I5" s="46"/>
-      <c r="J5" s="46" t="s">
+      <c r="J5" s="46"/>
+      <c r="K5" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="K5" s="46" t="s">
+      <c r="L5" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="L5" s="46" t="s">
+      <c r="M5" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="M5" s="46"/>
-      <c r="N5" s="46" t="s">
+      <c r="N5" s="46"/>
+      <c r="O5" s="46" t="s">
         <v>108</v>
       </c>
-      <c r="O5" s="47" t="s">
+      <c r="P5" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="P5" s="46" t="s">
+      <c r="Q5" s="46" t="s">
         <v>107</v>
       </c>
-      <c r="Q5" s="34" t="s">
+      <c r="R5" s="34" t="s">
         <v>110</v>
       </c>
-      <c r="R5" s="82" t="s">
+      <c r="S5" s="82" t="s">
         <v>112</v>
       </c>
-      <c r="S5" s="83"/>
       <c r="T5" s="83"/>
       <c r="U5" s="83"/>
       <c r="V5" s="83"/>
-      <c r="W5" s="35"/>
-      <c r="X5" s="84"/>
-      <c r="Y5" s="85"/>
+      <c r="W5" s="83"/>
+      <c r="X5" s="35"/>
+      <c r="Y5" s="84"/>
       <c r="Z5" s="85"/>
       <c r="AA5" s="85"/>
       <c r="AB5" s="85"/>
-      <c r="AC5" s="86"/>
+      <c r="AC5" s="85"/>
       <c r="AD5" s="86"/>
       <c r="AE5" s="86"/>
       <c r="AF5" s="86"/>
-      <c r="AG5" s="38" t="s">
+      <c r="AG5" s="86"/>
+      <c r="AH5" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="AH5" s="36"/>
-      <c r="AI5" s="37"/>
+      <c r="AI5" s="36"/>
       <c r="AJ5" s="37"/>
       <c r="AK5" s="37"/>
-      <c r="AL5" s="42" t="s">
+      <c r="AL5" s="37"/>
+      <c r="AM5" s="42" t="s">
         <v>105</v>
       </c>
-      <c r="AM5" s="43"/>
-      <c r="AN5" s="92"/>
+      <c r="AN5" s="43"/>
       <c r="AO5" s="92"/>
       <c r="AP5" s="92"/>
+      <c r="AQ5" s="92"/>
     </row>
-    <row r="6" spans="1:43" s="44" customFormat="1" ht="83.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:44" s="44" customFormat="1" ht="83.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="45" t="s">
         <v>98</v>
       </c>
@@ -2486,87 +2506,86 @@
       </c>
       <c r="F6" s="46"/>
       <c r="G6" s="46"/>
-      <c r="H6" s="46" t="s">
+      <c r="H6" s="46"/>
+      <c r="I6" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46" t="s">
+      <c r="J6" s="46"/>
+      <c r="K6" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="K6" s="46" t="s">
+      <c r="L6" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="L6" s="46"/>
-      <c r="M6" s="55"/>
-      <c r="N6" s="46"/>
-      <c r="O6" s="47"/>
-      <c r="P6" s="46"/>
-      <c r="Q6" s="48" t="s">
+      <c r="M6" s="46"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="46"/>
+      <c r="P6" s="47"/>
+      <c r="Q6" s="46"/>
+      <c r="R6" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="R6" s="104" t="s">
+      <c r="S6" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="S6" s="104"/>
       <c r="T6" s="104"/>
       <c r="U6" s="104"/>
       <c r="V6" s="104"/>
-      <c r="W6" s="49"/>
-      <c r="X6" s="50"/>
-      <c r="Y6" s="105" t="s">
+      <c r="W6" s="104"/>
+      <c r="X6" s="49"/>
+      <c r="Y6" s="50"/>
+      <c r="Z6" s="105" t="s">
         <v>43</v>
       </c>
-      <c r="Z6" s="105"/>
-      <c r="AA6" s="105" t="s">
+      <c r="AA6" s="105"/>
+      <c r="AB6" s="105" t="s">
         <v>44</v>
       </c>
-      <c r="AB6" s="105"/>
-      <c r="AC6" s="106"/>
+      <c r="AC6" s="105"/>
       <c r="AD6" s="106"/>
       <c r="AE6" s="106"/>
       <c r="AF6" s="106"/>
-      <c r="AG6" s="51"/>
-      <c r="AH6" s="100" t="s">
+      <c r="AG6" s="106"/>
+      <c r="AH6" s="51"/>
+      <c r="AI6" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="AI6" s="100"/>
-      <c r="AJ6" s="101" t="s">
+      <c r="AJ6" s="100"/>
+      <c r="AK6" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="AK6" s="101"/>
-      <c r="AL6" s="52"/>
-      <c r="AM6" s="53"/>
-      <c r="AN6" s="92"/>
+      <c r="AL6" s="101"/>
+      <c r="AM6" s="52"/>
+      <c r="AN6" s="53"/>
       <c r="AO6" s="92"/>
       <c r="AP6" s="92"/>
+      <c r="AQ6" s="92"/>
     </row>
-    <row r="7" spans="1:43" s="54" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:44" s="54" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="55"/>
       <c r="C7" s="55"/>
       <c r="D7" s="55"/>
       <c r="E7" s="55"/>
       <c r="F7" s="55"/>
       <c r="G7" s="55"/>
-      <c r="H7" s="55" t="s">
+      <c r="H7" s="55"/>
+      <c r="I7" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="55"/>
       <c r="J7" s="55"/>
       <c r="K7" s="55"/>
-      <c r="L7" s="55" t="s">
+      <c r="L7" s="55"/>
+      <c r="M7" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="55"/>
       <c r="N7" s="55"/>
-      <c r="O7" s="56"/>
-      <c r="P7" s="56" t="s">
+      <c r="O7" s="55"/>
+      <c r="P7" s="56"/>
+      <c r="Q7" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="58" t="s">
-        <v>47</v>
-      </c>
-      <c r="S7" s="59" t="s">
+      <c r="R7" s="57"/>
+      <c r="S7" s="58" t="s">
         <v>47</v>
       </c>
       <c r="T7" s="59" t="s">
@@ -2575,16 +2594,16 @@
       <c r="U7" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="V7" s="60" t="s">
+      <c r="V7" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="W7" s="61" t="s">
+      <c r="W7" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="X7" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="X7" s="64" t="s">
-        <v>46</v>
-      </c>
-      <c r="Y7" s="65" t="s">
+      <c r="Y7" s="64" t="s">
         <v>46</v>
       </c>
       <c r="Z7" s="65" t="s">
@@ -2593,13 +2612,13 @@
       <c r="AA7" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="AB7" s="66" t="s">
+      <c r="AB7" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="AC7" s="67" t="s">
+      <c r="AC7" s="66" t="s">
         <v>46</v>
       </c>
-      <c r="AD7" s="68" t="s">
+      <c r="AD7" s="67" t="s">
         <v>46</v>
       </c>
       <c r="AE7" s="68" t="s">
@@ -2608,23 +2627,26 @@
       <c r="AF7" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="AG7" s="69"/>
-      <c r="AH7" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI7" s="63" t="s">
+      <c r="AG7" s="68" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH7" s="69"/>
+      <c r="AI7" s="62" t="s">
         <v>48</v>
       </c>
       <c r="AJ7" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="AK7" s="70" t="s">
+      <c r="AK7" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="AL7" s="71"/>
-      <c r="AM7" s="72"/>
+      <c r="AL7" s="70" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM7" s="71"/>
+      <c r="AN7" s="72"/>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>49</v>
       </c>
@@ -2637,66 +2659,66 @@
       <c r="E8" t="s">
         <v>61</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>58</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>10</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>5</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>1</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>3600</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>59</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>95</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>60</v>
       </c>
-      <c r="Q8" s="2" t="s">
+      <c r="R8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R8" s="1">
+      <c r="S8" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <v>424.4298</v>
       </c>
-      <c r="X8" s="1">
+      <c r="Y8" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y8" s="5">
+      <c r="Z8" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z8" s="4">
+      <c r="AA8" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG8" s="1">
+      <c r="AH8" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH8" s="1">
+      <c r="AI8" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI8">
+      <c r="AJ8">
         <v>383.476</v>
       </c>
-      <c r="AK8" s="73"/>
-      <c r="AL8" s="2">
+      <c r="AL8" s="73"/>
+      <c r="AM8" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
@@ -2709,65 +2731,65 @@
       <c r="E9" t="s">
         <v>62</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>57</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>58</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>10</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>5</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>1</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>3600</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>59</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>96</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>60</v>
       </c>
-      <c r="Q9" s="2" t="s">
+      <c r="R9" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R9" s="1">
+      <c r="S9" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <v>424.4298</v>
       </c>
-      <c r="X9" s="1">
+      <c r="Y9" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y9" s="5">
+      <c r="Z9" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z9" s="4">
+      <c r="AA9" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG9" s="1">
+      <c r="AH9" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH9" s="1">
+      <c r="AI9" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI9">
+      <c r="AJ9">
         <v>383.476</v>
       </c>
-      <c r="AL9" s="2">
+      <c r="AM9" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>49</v>
       </c>
@@ -2780,65 +2802,65 @@
       <c r="E10" t="s">
         <v>63</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>57</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>58</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>10</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>5</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>1</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>3600</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>59</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>97</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>60</v>
       </c>
-      <c r="Q10" s="2" t="s">
+      <c r="R10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R10" s="1">
+      <c r="S10" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <v>424.4298</v>
       </c>
-      <c r="X10" s="1">
+      <c r="Y10" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y10" s="5">
+      <c r="Z10" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z10" s="4">
+      <c r="AA10" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG10" s="1">
+      <c r="AH10" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH10" s="1">
+      <c r="AI10" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI10">
+      <c r="AJ10">
         <v>383.476</v>
       </c>
-      <c r="AL10" s="2">
+      <c r="AM10" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>49</v>
       </c>
@@ -2851,65 +2873,65 @@
       <c r="E11" t="s">
         <v>64</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>57</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>58</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>10</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>5</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>1</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>3600</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>59</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>95</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>75</v>
       </c>
-      <c r="Q11" s="2" t="s">
+      <c r="R11" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R11" s="1">
+      <c r="S11" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W11">
+      <c r="X11">
         <v>424.4298</v>
       </c>
-      <c r="X11" s="1">
+      <c r="Y11" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y11" s="5">
+      <c r="Z11" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z11" s="4">
+      <c r="AA11" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG11" s="1">
+      <c r="AH11" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH11" s="1">
+      <c r="AI11" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI11">
+      <c r="AJ11">
         <v>383.476</v>
       </c>
-      <c r="AL11" s="2">
+      <c r="AM11" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>49</v>
       </c>
@@ -2922,68 +2944,68 @@
       <c r="E12" t="s">
         <v>65</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>57</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>58</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>10</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>5</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>1</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>3600</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>59</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>96</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>75</v>
       </c>
-      <c r="Q12" s="2" t="s">
+      <c r="R12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R12" s="1">
+      <c r="S12" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W12">
+      <c r="X12">
         <v>424.4298</v>
       </c>
-      <c r="X12" s="1">
+      <c r="Y12" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y12" s="5">
+      <c r="Z12" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z12" s="4">
+      <c r="AA12" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG12" s="1">
+      <c r="AH12" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH12" s="1">
+      <c r="AI12" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI12">
+      <c r="AJ12">
         <v>383.476</v>
       </c>
-      <c r="AJ12" t="s">
+      <c r="AK12" t="s">
         <v>52</v>
       </c>
-      <c r="AL12" s="2">
+      <c r="AM12" s="2">
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:44" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>49</v>
       </c>
@@ -2996,79 +3018,79 @@
       <c r="E13" t="s">
         <v>66</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>57</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>58</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>10</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>5</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>1</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>3600</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>59</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>97</v>
       </c>
-      <c r="P13">
+      <c r="Q13">
         <v>75</v>
       </c>
-      <c r="Q13" s="2" t="s">
+      <c r="R13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R13" s="1">
+      <c r="S13" s="1">
         <v>349.83049999999997</v>
       </c>
-      <c r="W13">
+      <c r="X13">
         <v>424.4298</v>
       </c>
-      <c r="X13" s="1">
+      <c r="Y13" s="1">
         <v>59.0717</v>
       </c>
-      <c r="Y13" s="5">
+      <c r="Z13" s="5">
         <v>56.555799999999998</v>
       </c>
-      <c r="Z13" s="4">
+      <c r="AA13" s="4">
         <v>59.491</v>
       </c>
-      <c r="AG13" s="1">
+      <c r="AH13" s="1">
         <v>0.9</v>
       </c>
-      <c r="AH13" s="1">
+      <c r="AI13" s="1">
         <v>498.89100000000002</v>
       </c>
-      <c r="AI13">
+      <c r="AJ13">
         <v>383.476</v>
       </c>
-      <c r="AL13" s="2">
+      <c r="AM13" s="2">
         <v>106</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="AH2:AK2"/>
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="R1:AF1"/>
-    <mergeCell ref="R2:AF2"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="X4:AB4"/>
-    <mergeCell ref="AC4:AF4"/>
-    <mergeCell ref="R6:V6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="AC6:AF6"/>
-    <mergeCell ref="R4:V4"/>
+    <mergeCell ref="AI2:AL2"/>
+    <mergeCell ref="AI1:AL1"/>
+    <mergeCell ref="S1:AG1"/>
+    <mergeCell ref="S2:AG2"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="Y4:AC4"/>
+    <mergeCell ref="AD4:AG4"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AD6:AG6"/>
+    <mergeCell ref="S4:W4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
@@ -3084,49 +3106,49 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="88" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="74" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="74" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="74" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="74" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="89" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>119</v>
       </c>

</xml_diff>